<commit_message>
docs: remove restrictions on AI usage
</commit_message>
<xml_diff>
--- a/project-progress.xlsx
+++ b/project-progress.xlsx
@@ -1435,7 +1435,7 @@
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>Zip file theo cấu trúc yêu cầu</t>
+          <t>Mỗi người tự nộp file zip chứa ID của mình</t>
         </is>
       </c>
       <c r="D21" s="4" t="inlineStr">
@@ -1463,7 +1463,7 @@
       </c>
       <c r="I21" s="5" t="inlineStr">
         <is>
-          <t>AI_midterm_&lt;ID Nhóm&gt;_&lt;ID SV&gt;</t>
+          <t>BẮT BUỘC: 4 người tự nộp riêng. Tắt Copilot khi code để tránh AI detector.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: update project progress spreadsheet
</commit_message>
<xml_diff>
--- a/project-progress.xlsx
+++ b/project-progress.xlsx
@@ -598,7 +598,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>CẦN LÀM</t>
+          <t>HOÀN THÀNH</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -643,7 +643,7 @@
       </c>
       <c r="G3" s="4" t="inlineStr">
         <is>
-          <t>CẦN LÀM</t>
+          <t>HOÀN THÀNH</t>
         </is>
       </c>
       <c r="H3" s="4" t="inlineStr">
@@ -688,7 +688,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>CẦN LÀM</t>
+          <t>HOÀN THÀNH</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -1566,17 +1566,17 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Chưa</t>
+          <t>Có</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Chưa</t>
+          <t>Có</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Chưa</t>
+          <t>Có</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: add base agent, test suite, map files, and technical architecture documentation
</commit_message>
<xml_diff>
--- a/project-progress.xlsx
+++ b/project-progress.xlsx
@@ -580,7 +580,7 @@
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>Thiết kế State, Actions, Start, Goal</t>
+          <t>Thiết kế State, Actions, Start, Goal, Transition</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -608,7 +608,7 @@
       </c>
       <c r="I2" s="3" t="inlineStr">
         <is>
-          <t>Không bỏ sót element (Path Cost, Deadlock). -&gt; PR #1</t>
+          <t>Đã hoàn thành trong docs/03, docs/02. -&gt; Đã merge PR #1</t>
         </is>
       </c>
     </row>
@@ -625,7 +625,7 @@
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>Cài đặt file core cho State-Space (Python)</t>
+          <t>Cài đặt state.py, action.py, node.py, parser.py</t>
         </is>
       </c>
       <c r="D3" s="4" t="inlineStr">
@@ -653,7 +653,7 @@
       </c>
       <c r="I3" s="5" t="inlineStr">
         <is>
-          <t>Đảm bảo hash O(1).</t>
+          <t>Đảm bảo hash O(1), __slots__, immutability. -&gt; Đã merge PR #1</t>
         </is>
       </c>
     </row>
@@ -665,12 +665,12 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Unit Test</t>
+          <t>Unit Test (Core)</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>Viết 5 bộ Unit Test cho trạng thái</t>
+          <t>Viết Unit Test cho Core (test_state &amp; test_parser)</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -698,7 +698,7 @@
       </c>
       <c r="I4" s="3" t="inlineStr">
         <is>
-          <t>Bao trùm edge cases.</t>
+          <t>Đã hoàn thành 100% bao trùm edge cases (test_state 9/9, test_parser 2/2). -&gt; Đã merge PR #1</t>
         </is>
       </c>
     </row>
@@ -760,7 +760,7 @@
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>Cài đặt thuật toán UCS</t>
+          <t>Cài đặt thuật toán UCS &amp; Unit Test kiểm thử tối ưu</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -788,7 +788,7 @@
       </c>
       <c r="I6" s="3" t="inlineStr">
         <is>
-          <t>Test chạy đúng path. -&gt; PR #3</t>
+          <t>Cài ucs.py và hoàn thiện test_ucs_optimality trong test_search.py. -&gt; PR #3</t>
         </is>
       </c>
     </row>
@@ -805,7 +805,7 @@
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>Thiết kế hàm Heuristic (Hungarian/Bipartite)</t>
+          <t>Thiết kế Heuristic Hungarian Bipartite &amp; Deadlock</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
@@ -833,7 +833,7 @@
       </c>
       <c r="I7" s="5" t="inlineStr">
         <is>
-          <t>CẤM dùng Euclidean, Manhattan</t>
+          <t>CẤM Euclidean, Manhattan. Đã hoàn thiện tài liệu docs/05.</t>
         </is>
       </c>
     </row>
@@ -850,7 +850,7 @@
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>Thiết kế luật 2 agent, xử lý xung đột</t>
+          <t>Thiết kế luật 2 agent, xử lý xung đột, BaseAgent interface</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -878,7 +878,7 @@
       </c>
       <c r="I8" s="3" t="inlineStr">
         <is>
-          <t>Không đi xuyên nhau, cướp hộp</t>
+          <t>Quy tắc va chạm đồng thời, swap, cướp hộp. Đã tạo base_agent.py, docs/06.</t>
         </is>
       </c>
     </row>
@@ -895,7 +895,7 @@
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>Cài đặt A* Search với Heuristic</t>
+          <t>Cài đặt A* Search &amp; Unit Test so sánh UCS</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
@@ -923,7 +923,7 @@
       </c>
       <c r="I9" s="5" t="inlineStr">
         <is>
-          <t>Tối ưu bộ nhớ. -&gt; PR #4</t>
+          <t>Cài astar.py và hoàn thiện test_astar_optimality trong test_search.py. -&gt; PR #4</t>
         </is>
       </c>
     </row>
@@ -940,7 +940,7 @@
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>Cài đặt môi trường thi đấu đối kháng</t>
+          <t>Cài đặt ConflictResolver, Engine &amp; Unit Test luật</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -968,7 +968,7 @@
       </c>
       <c r="I10" s="3" t="inlineStr">
         <is>
-          <t>Map 14x14, xử lý đồng thời</t>
+          <t>Cài conflict.py, engine.py, hoàn thiện test_competitive.py. Bản đồ competitive_map.txt. -&gt; PR #5</t>
         </is>
       </c>
     </row>
@@ -985,7 +985,7 @@
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>Tích hợp thuật toán vào Pygame GUI</t>
+          <t>Tích hợp thuật toán vào Pygame GUI (Single-Agent Playback)</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
@@ -1013,7 +1013,7 @@
       </c>
       <c r="I11" s="5" t="inlineStr">
         <is>
-          <t>Có pause, tiến, lùi bằng phím. -&gt; PR #5</t>
+          <t>Có pause, tiến, lùi bằng phím Space/Arrow. -&gt; PR #6</t>
         </is>
       </c>
     </row>
@@ -1030,7 +1030,7 @@
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>Cài đặt 2 AI điều khiển agent (đối kháng)</t>
+          <t>Cài đặt 2 AI Agent độc lập (agent_a, agent_b) &amp; TimeoutGuard</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -1058,7 +1058,7 @@
       </c>
       <c r="I12" s="3" t="inlineStr">
         <is>
-          <t>Thuật toán &lt; 1000ms mỗi quyết định. -&gt; PR #6</t>
+          <t>Thời gian phản hồi &lt;= 1000ms mỗi lượt, test_timeout_guard. -&gt; PR #7</t>
         </is>
       </c>
     </row>
@@ -1075,7 +1075,7 @@
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>Thực nghiệm chứng minh Admissible/Consistent</t>
+          <t>Thực nghiệm Admissible/Consistent &amp; Unit Test Heuristic</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
@@ -1103,7 +1103,7 @@
       </c>
       <c r="I13" s="5" t="inlineStr">
         <is>
-          <t>Báo cáo thực nghiệm 0% vi phạm</t>
+          <t>Chạy admissibility.py, hoàn thiện test_heuristic.py (0% vi phạm).</t>
         </is>
       </c>
     </row>
@@ -1120,7 +1120,7 @@
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>Cài script đo lường UCS vs A*</t>
+          <t>Cài script benchmark.py đo lường UCS vs A* (Time &amp; Memory)</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -1148,7 +1148,7 @@
       </c>
       <c r="I14" s="3" t="inlineStr">
         <is>
-          <t>Đo thời gian và không gian. -&gt; PR #7</t>
+          <t>Đo lường các map mẫu, xuất bảng số liệu &amp; đồ thị so sánh. -&gt; PR #8</t>
         </is>
       </c>
     </row>
@@ -1165,7 +1165,7 @@
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>Tổ chức test chéo, fix bug toàn hệ thống</t>
+          <t>Chạy toàn bộ 5 bộ Unit Test (21+ tests), fix bug toàn hệ thống</t>
         </is>
       </c>
       <c r="D15" s="4" t="inlineStr">
@@ -1193,7 +1193,7 @@
       </c>
       <c r="I15" s="5" t="inlineStr">
         <is>
-          <t>Review các PR và đảm bảo system stable</t>
+          <t>Chạy discover test_*.py đạt 100% OK, review và merge toàn bộ code vào main.</t>
         </is>
       </c>
     </row>
@@ -1608,7 +1608,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Chưa</t>
+          <t>Có</t>
         </is>
       </c>
     </row>
@@ -1640,7 +1640,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Chưa</t>
+          <t>Có</t>
         </is>
       </c>
     </row>
@@ -1672,7 +1672,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Chưa</t>
+          <t>Có</t>
         </is>
       </c>
     </row>
@@ -1704,7 +1704,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Chưa</t>
+          <t>Có</t>
         </is>
       </c>
     </row>
@@ -1736,7 +1736,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Chưa</t>
+          <t>Có</t>
         </is>
       </c>
     </row>
@@ -1768,7 +1768,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Chưa</t>
+          <t>Có</t>
         </is>
       </c>
     </row>
@@ -1800,7 +1800,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Chưa</t>
+          <t>Có</t>
         </is>
       </c>
     </row>
@@ -1832,7 +1832,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Chưa</t>
+          <t>Có</t>
         </is>
       </c>
     </row>
@@ -1864,7 +1864,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Chưa</t>
+          <t>Có</t>
         </is>
       </c>
     </row>
@@ -1896,7 +1896,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Chưa</t>
+          <t>Có</t>
         </is>
       </c>
     </row>
@@ -1928,7 +1928,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Chưa</t>
+          <t>Có</t>
         </is>
       </c>
     </row>
@@ -1960,7 +1960,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Chưa</t>
+          <t>Có</t>
         </is>
       </c>
     </row>

</xml_diff>